<commit_message>
adding rest of the assignment files to commit. there was a large file and I tried to remove it from commit history but then it make the assignment-3 and main branches have separate histories and be unable to merge. so then I changed the history of main to match the history of assignment-3, but then that made the branches identical so there was nothing to merge. So I made some slight edits to the assignment files so they show up in the commit.
</commit_message>
<xml_diff>
--- a/assignment_3_files/DSI_vis_assignment_3_cpi.xlsx
+++ b/assignment_3_files/DSI_vis_assignment_3_cpi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robertlu/Documents/Biochemistry/DSI/visualization/assignment_3_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52CA3C9B-D59A-824F-9405-2733EBB7BBE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98105A77-BABF-5E48-8F26-7C0583A17904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30240" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6803,7 +6803,7 @@
           <c:yMode val="edge"/>
           <c:x val="0.10343735137134703"/>
           <c:y val="0.11215018305832788"/>
-          <c:w val="0.663218009563873"/>
+          <c:w val="0.73033213549648579"/>
           <c:h val="0.21269058127288229"/>
         </c:manualLayout>
       </c:layout>
@@ -6820,7 +6820,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>

</xml_diff>